<commit_message>
UK daily ratings for 2026-05-03
</commit_message>
<xml_diff>
--- a/output/daily_ratings/uk_ratings_2026-05-03.xlsx
+++ b/output/daily_ratings/uk_ratings_2026-05-03.xlsx
@@ -1212,17 +1212,17 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Trek Home (IRE)</t>
+          <t>Xerling (IRE)</t>
         </is>
       </c>
       <c r="I14" t="n">
         <v>3</v>
       </c>
       <c r="J14" t="n">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>78</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
@@ -1266,17 +1266,17 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Xerling (IRE)</t>
+          <t>The Pipers Call (IRE)</t>
         </is>
       </c>
       <c r="I15" t="n">
         <v>3</v>
       </c>
       <c r="J15" t="n">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="K15" t="n">
-        <v>78</v>
+        <v>0</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
@@ -1320,7 +1320,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>The Pipers Call (IRE)</t>
+          <t>Trek Home (IRE)</t>
         </is>
       </c>
       <c r="I16" t="n">
@@ -2242,17 +2242,17 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Aviatrice (IRE)</t>
+          <t>Nancy J (IRE)</t>
         </is>
       </c>
       <c r="I32" t="n">
         <v>4</v>
       </c>
       <c r="J32" t="n">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K32" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="n">
@@ -2296,17 +2296,17 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Nancy J (IRE)</t>
+          <t>Aviatrice (IRE)</t>
         </is>
       </c>
       <c r="I33" t="n">
         <v>4</v>
       </c>
       <c r="J33" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K33" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="n">
@@ -3614,17 +3614,17 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>Truth Be Told (IRE)</t>
+          <t>Alba Chiara (IRE)</t>
         </is>
       </c>
       <c r="I56" t="n">
         <v>4</v>
       </c>
       <c r="J56" t="n">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="K56" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="L56" t="inlineStr"/>
       <c r="M56" t="n">
@@ -3668,17 +3668,17 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Happy Pharoah (IRE)</t>
+          <t>Genoah (IRE)</t>
         </is>
       </c>
       <c r="I57" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J57" t="n">
-        <v>144</v>
+        <v>120</v>
       </c>
       <c r="K57" t="n">
-        <v>104</v>
+        <v>80</v>
       </c>
       <c r="L57" t="inlineStr"/>
       <c r="M57" t="n">
@@ -3722,17 +3722,17 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>Alba Chiara (IRE)</t>
+          <t>Truth Be Told (IRE)</t>
         </is>
       </c>
       <c r="I58" t="n">
         <v>4</v>
       </c>
       <c r="J58" t="n">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="K58" t="n">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="L58" t="inlineStr"/>
       <c r="M58" t="n">
@@ -3776,17 +3776,17 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Genoah (IRE)</t>
+          <t>Happy Pharoah (IRE)</t>
         </is>
       </c>
       <c r="I59" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J59" t="n">
-        <v>120</v>
+        <v>144</v>
       </c>
       <c r="K59" t="n">
-        <v>80</v>
+        <v>104</v>
       </c>
       <c r="L59" t="inlineStr"/>
       <c r="M59" t="n">
@@ -5314,7 +5314,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>Themis (IRE)</t>
+          <t>Zitkala Sa (IRE)</t>
         </is>
       </c>
       <c r="I86" t="n">
@@ -5368,7 +5368,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>Zitkala Sa (IRE)</t>
+          <t>Lake Bonney (IRE)</t>
         </is>
       </c>
       <c r="I87" t="n">
@@ -5422,7 +5422,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>Lake Bonney (IRE)</t>
+          <t>Themis (IRE)</t>
         </is>
       </c>
       <c r="I88" t="n">
@@ -6054,7 +6054,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>Sunrush (IRE)</t>
+          <t>Maxminelli (IRE)</t>
         </is>
       </c>
       <c r="I99" t="n">
@@ -6064,7 +6064,7 @@
         <v>132</v>
       </c>
       <c r="K99" t="n">
-        <v>0</v>
+        <v>69</v>
       </c>
       <c r="L99" t="inlineStr"/>
       <c r="M99" t="n">
@@ -6108,17 +6108,17 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>Maxminelli (IRE)</t>
+          <t>Roi Du Nord (IRE)</t>
         </is>
       </c>
       <c r="I100" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J100" t="n">
-        <v>132</v>
+        <v>147</v>
       </c>
       <c r="K100" t="n">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="L100" t="inlineStr"/>
       <c r="M100" t="n">
@@ -6162,14 +6162,14 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>Roi Du Nord (IRE)</t>
+          <t>Sunrush (IRE)</t>
         </is>
       </c>
       <c r="I101" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J101" t="n">
-        <v>147</v>
+        <v>132</v>
       </c>
       <c r="K101" t="n">
         <v>0</v>
@@ -16604,17 +16604,17 @@
       </c>
       <c r="H277" t="inlineStr">
         <is>
-          <t>Calshot Spit (IRE)</t>
+          <t>High Favour (IRE)</t>
         </is>
       </c>
       <c r="I277" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J277" t="n">
-        <v>130</v>
+        <v>116</v>
       </c>
       <c r="K277" t="n">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="L277" t="inlineStr"/>
       <c r="M277" t="n">
@@ -16660,17 +16660,17 @@
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>Beggarman</t>
+          <t>Kotari (FR)</t>
         </is>
       </c>
       <c r="I278" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J278" t="n">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="K278" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="L278" t="inlineStr"/>
       <c r="M278" t="n">
@@ -16716,17 +16716,17 @@
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t>High Favour (IRE)</t>
+          <t>Calshot Spit (IRE)</t>
         </is>
       </c>
       <c r="I279" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J279" t="n">
-        <v>116</v>
+        <v>130</v>
       </c>
       <c r="K279" t="n">
-        <v>46</v>
+        <v>60</v>
       </c>
       <c r="L279" t="inlineStr"/>
       <c r="M279" t="n">
@@ -16772,17 +16772,17 @@
       </c>
       <c r="H280" t="inlineStr">
         <is>
-          <t>Kotari (FR)</t>
+          <t>Beggarman</t>
         </is>
       </c>
       <c r="I280" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J280" t="n">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="K280" t="n">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="L280" t="inlineStr"/>
       <c r="M280" t="n">
@@ -20458,17 +20458,17 @@
       </c>
       <c r="H344" t="inlineStr">
         <is>
-          <t>Copper Craft (IRE)</t>
+          <t>Cleopatras Needle (IRE)</t>
         </is>
       </c>
       <c r="I344" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J344" t="n">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="K344" t="n">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="L344" t="inlineStr"/>
       <c r="M344" t="n">
@@ -20512,17 +20512,17 @@
       </c>
       <c r="H345" t="inlineStr">
         <is>
-          <t>Cleopatras Needle (IRE)</t>
+          <t>Copper Craft (IRE)</t>
         </is>
       </c>
       <c r="I345" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J345" t="n">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="K345" t="n">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="L345" t="inlineStr"/>
       <c r="M345" t="n">

</xml_diff>